<commit_message>
Slice D2: Adjudicator Information Sheet milestone fill + golden re-bless (#87)
Render each judge's contracting milestones on the Adjudicator Information
Sheet (.xlsx) via D1's shared adjudicatorMilestoneStatus derivation: a
completed milestone shows a check + its stored date (the sheet's existing
fmtDate formatter), a pending one shows "pending" — a snapshot as of
generation. Existing power/hotel/dietary needs are unchanged.

The builder reads only stored milestone dates (never the clock), so output
stays deterministic. Fixture judges now carry a deliberate mix — judge 1 all
done (distinct dates), judge 2 partly done, judge 3 all pending — so the
re-blessed golden exercises both the check-with-date and "pending" paths.

No other document or registry change.

Closes #87.
</commit_message>
<xml_diff>
--- a/app/src/documents/__fixtures__/golden/Adjudicator Info Sheet.xlsx
+++ b/app/src/documents/__fixtures__/golden/Adjudicator Info Sheet.xlsx
@@ -409,7 +409,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C30"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -508,52 +508,151 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="str">
-        <v>Judge 2</v>
+        <v>Contracting</v>
       </c>
       <c r="B15" s="2" t="str">
-        <v>Prof. John Critic</v>
+        <v>✓ TTAO contract: Sunday, February 15, 2026</v>
       </c>
       <c r="C15" s="2" t="str">
-        <v>200 Oak Ave, Dallas, TX 75201</v>
+        <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="str">
-        <v>Judge 3</v>
+        <v/>
       </c>
       <c r="B16" s="2" t="str">
-        <v>Ms. Mary Adjudicator</v>
+        <v>✓ Payment paperwork sent: Sunday, March 1, 2026</v>
       </c>
       <c r="C16" s="2" t="str">
-        <v>300 Elm Blvd, San Antonio, TX 78205</v>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B17" s="2" t="str">
+        <v>✓ Payment paperwork returned: Tuesday, March 10, 2026</v>
+      </c>
+      <c r="C17" s="2" t="str">
+        <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="str">
-        <v>CONTEST MANAGER</v>
+        <v>Judge 2</v>
+      </c>
+      <c r="B18" s="2" t="str">
+        <v>Prof. John Critic</v>
+      </c>
+      <c r="C18" s="2" t="str">
+        <v>200 Oak Ave, Dallas, TX 75201</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="str">
-        <v>Name</v>
+        <v>Contracting</v>
       </c>
       <c r="B19" s="2" t="str">
-        <v>Allen Otto</v>
+        <v>✓ TTAO contract: Friday, February 20, 2026</v>
+      </c>
+      <c r="C19" s="2" t="str">
+        <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="str">
-        <v>Email</v>
+        <v/>
       </c>
       <c r="B20" s="2" t="str">
-        <v>aotto3@gmail.com</v>
+        <v>✓ Payment paperwork sent: Thursday, March 5, 2026</v>
+      </c>
+      <c r="C20" s="2" t="str">
+        <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B21" s="2" t="str">
+        <v>Payment paperwork returned: pending</v>
+      </c>
+      <c r="C21" s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="str">
+        <v>Judge 3</v>
+      </c>
+      <c r="B22" s="2" t="str">
+        <v>Ms. Mary Adjudicator</v>
+      </c>
+      <c r="C22" s="2" t="str">
+        <v>300 Elm Blvd, San Antonio, TX 78205</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="str">
+        <v>Contracting</v>
+      </c>
+      <c r="B23" s="2" t="str">
+        <v>TTAO contract: pending</v>
+      </c>
+      <c r="C23" s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B24" s="2" t="str">
+        <v>Payment paperwork sent: pending</v>
+      </c>
+      <c r="C24" s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B25" s="2" t="str">
+        <v>Payment paperwork returned: pending</v>
+      </c>
+      <c r="C25" s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="str">
+        <v>CONTEST MANAGER</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="str">
+        <v>Name</v>
+      </c>
+      <c r="B28" s="2" t="str">
+        <v>Allen Otto</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="str">
+        <v>Email</v>
+      </c>
+      <c r="B29" s="2" t="str">
+        <v>aotto3@gmail.com</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="str">
         <v>Phone</v>
       </c>
-      <c r="B21" s="2" t="str">
+      <c r="B30" s="2" t="str">
         <v>281-777-8672</v>
       </c>
     </row>
@@ -563,7 +662,7 @@
     <mergeCell ref="A2:C2"/>
   </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C30"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Slice D2: Adjudicator Information Sheet milestone fill + golden re-bless (#87) (#110)
Render each judge's contracting milestones on the Adjudicator Information
Sheet (.xlsx) via D1's shared adjudicatorMilestoneStatus derivation: a
completed milestone shows a check + its stored date (the sheet's existing
fmtDate formatter), a pending one shows "pending" — a snapshot as of
generation. Existing power/hotel/dietary needs are unchanged.

The builder reads only stored milestone dates (never the clock), so output
stays deterministic. Fixture judges now carry a deliberate mix — judge 1 all
done (distinct dates), judge 2 partly done, judge 3 all pending — so the
re-blessed golden exercises both the check-with-date and "pending" paths.

No other document or registry change.

Closes #87.
</commit_message>
<xml_diff>
--- a/app/src/documents/__fixtures__/golden/Adjudicator Info Sheet.xlsx
+++ b/app/src/documents/__fixtures__/golden/Adjudicator Info Sheet.xlsx
@@ -409,7 +409,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C30"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -508,52 +508,151 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="str">
-        <v>Judge 2</v>
+        <v>Contracting</v>
       </c>
       <c r="B15" s="2" t="str">
-        <v>Prof. John Critic</v>
+        <v>✓ TTAO contract: Sunday, February 15, 2026</v>
       </c>
       <c r="C15" s="2" t="str">
-        <v>200 Oak Ave, Dallas, TX 75201</v>
+        <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="str">
-        <v>Judge 3</v>
+        <v/>
       </c>
       <c r="B16" s="2" t="str">
-        <v>Ms. Mary Adjudicator</v>
+        <v>✓ Payment paperwork sent: Sunday, March 1, 2026</v>
       </c>
       <c r="C16" s="2" t="str">
-        <v>300 Elm Blvd, San Antonio, TX 78205</v>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B17" s="2" t="str">
+        <v>✓ Payment paperwork returned: Tuesday, March 10, 2026</v>
+      </c>
+      <c r="C17" s="2" t="str">
+        <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="str">
-        <v>CONTEST MANAGER</v>
+        <v>Judge 2</v>
+      </c>
+      <c r="B18" s="2" t="str">
+        <v>Prof. John Critic</v>
+      </c>
+      <c r="C18" s="2" t="str">
+        <v>200 Oak Ave, Dallas, TX 75201</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="str">
-        <v>Name</v>
+        <v>Contracting</v>
       </c>
       <c r="B19" s="2" t="str">
-        <v>Allen Otto</v>
+        <v>✓ TTAO contract: Friday, February 20, 2026</v>
+      </c>
+      <c r="C19" s="2" t="str">
+        <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="str">
-        <v>Email</v>
+        <v/>
       </c>
       <c r="B20" s="2" t="str">
-        <v>aotto3@gmail.com</v>
+        <v>✓ Payment paperwork sent: Thursday, March 5, 2026</v>
+      </c>
+      <c r="C20" s="2" t="str">
+        <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B21" s="2" t="str">
+        <v>Payment paperwork returned: pending</v>
+      </c>
+      <c r="C21" s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="str">
+        <v>Judge 3</v>
+      </c>
+      <c r="B22" s="2" t="str">
+        <v>Ms. Mary Adjudicator</v>
+      </c>
+      <c r="C22" s="2" t="str">
+        <v>300 Elm Blvd, San Antonio, TX 78205</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="str">
+        <v>Contracting</v>
+      </c>
+      <c r="B23" s="2" t="str">
+        <v>TTAO contract: pending</v>
+      </c>
+      <c r="C23" s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B24" s="2" t="str">
+        <v>Payment paperwork sent: pending</v>
+      </c>
+      <c r="C24" s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B25" s="2" t="str">
+        <v>Payment paperwork returned: pending</v>
+      </c>
+      <c r="C25" s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="str">
+        <v>CONTEST MANAGER</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="str">
+        <v>Name</v>
+      </c>
+      <c r="B28" s="2" t="str">
+        <v>Allen Otto</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="str">
+        <v>Email</v>
+      </c>
+      <c r="B29" s="2" t="str">
+        <v>aotto3@gmail.com</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="str">
         <v>Phone</v>
       </c>
-      <c r="B21" s="2" t="str">
+      <c r="B30" s="2" t="str">
         <v>281-777-8672</v>
       </c>
     </row>
@@ -563,7 +662,7 @@
     <mergeCell ref="A2:C2"/>
   </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C30"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>